<commit_message>
Fix prijzen homepage, netto verwijderen, VVS logo header, DB updates
- ProjectCard: prijsbadge toont nu volledige prijs (€ + bedrag) i.p.v. alleen €
- ProjectModal: tabel toont alleen bruto oppervlakte, netto kolommen verwijderd
- Bedrijfsunit detail page: alleen bruto tonen, 2e verdieping dynamisch berekend en getoond voor units 1, 12, 57
- Bedrijfsunit listing tabel: industrie/kantoor kolommen tonen nu bruto i.p.v. netto
- Header: VVS Projectontwikkeling logo toegevoegd naast bestaand logo (alleen desktop)
- DB: opslagbox unit 14 status op 'reserved' gezet

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/brutonetto bedrijfspand inc. verkoopprijs.xlsx
+++ b/brutonetto bedrijfspand inc. verkoopprijs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/26298b6f56744992/Desktop/project de steiger/de steiger/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vireshkewalbansing/Repos/unity-units-clone/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="8_{215E58DF-5135-40E2-B608-8823AE995B5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FB98551-60CA-4BC7-92A7-2B2123D26791}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7AD1A26-D1C2-7D4C-BD64-1FECB132EE63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -157,8 +157,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="44" formatCode="_ &quot;€&quot;\ * #,##0.00_ ;_ &quot;€&quot;\ * \-#,##0.00_ ;_ &quot;€&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="164" formatCode="_ [$€-413]\ * #.##0.00_ ;_ [$€-413]\ * \-#.##0.00_ ;_ [$€-413]\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_ &quot;€&quot;\ * #,##0.00_ ;_ &quot;€&quot;\ * \-#,##0.00_ ;_ &quot;€&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_ [$€-413]\ * #.##0.00_ ;_ [$€-413]\ * \-#.##0.00_ ;_ [$€-413]\ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -468,7 +468,7 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="83">
@@ -514,14 +514,86 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -612,12 +684,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -631,72 +697,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1061,272 +1061,273 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:W96"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.33203125" customWidth="1"/>
     <col min="2" max="7" width="7.6640625" customWidth="1"/>
-    <col min="8" max="8" width="0.88671875" customWidth="1"/>
+    <col min="8" max="8" width="0.83203125" customWidth="1"/>
     <col min="9" max="14" width="7.6640625" customWidth="1"/>
-    <col min="15" max="15" width="0.88671875" customWidth="1"/>
+    <col min="15" max="15" width="0.83203125" customWidth="1"/>
     <col min="16" max="17" width="9.6640625" customWidth="1"/>
     <col min="18" max="18" width="7.33203125" customWidth="1"/>
-    <col min="19" max="19" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.44140625" customWidth="1"/>
+    <col min="19" max="19" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.5" customWidth="1"/>
     <col min="21" max="21" width="21.6640625" customWidth="1"/>
-    <col min="22" max="22" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="19.33203125" customWidth="1"/>
+    <col min="23" max="23" width="10.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="30" t="s">
+    <row r="1" spans="1:22" ht="24" x14ac:dyDescent="0.3">
+      <c r="A1" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="31" t="s">
+      <c r="B1" s="54"/>
+      <c r="C1" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-    </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55"/>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A2" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="32" t="s">
+      <c r="B2" s="54"/>
+      <c r="C2" s="56" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
+      <c r="L2" s="56"/>
+      <c r="M2" s="56"/>
+      <c r="N2" s="56"/>
       <c r="O2" s="3"/>
     </row>
-    <row r="3" spans="1:22" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="30" t="s">
+    <row r="3" spans="1:22" ht="19" x14ac:dyDescent="0.25">
+      <c r="A3" s="54" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="33" t="s">
+      <c r="B3" s="54"/>
+      <c r="C3" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
-      <c r="J3" s="33"/>
-      <c r="K3" s="33"/>
-      <c r="L3" s="33"/>
-      <c r="M3" s="33"/>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A4" s="30" t="s">
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="57"/>
+      <c r="L3" s="57"/>
+      <c r="M3" s="57"/>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A4" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="34">
+      <c r="B4" s="54"/>
+      <c r="C4" s="58">
         <v>45762</v>
       </c>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="34"/>
-      <c r="M4" s="34"/>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58"/>
+      <c r="J4" s="58"/>
+      <c r="K4" s="58"/>
+      <c r="L4" s="58"/>
+      <c r="M4" s="58"/>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="R5" s="2"/>
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A6" s="56" t="s">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A6" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="57"/>
-      <c r="C6" s="57"/>
-      <c r="D6" s="57"/>
-      <c r="E6" s="57"/>
-      <c r="F6" s="57"/>
-      <c r="G6" s="57"/>
-      <c r="H6" s="57"/>
-      <c r="I6" s="57"/>
-      <c r="J6" s="57"/>
-      <c r="K6" s="58"/>
+      <c r="B6" s="79"/>
+      <c r="C6" s="79"/>
+      <c r="D6" s="79"/>
+      <c r="E6" s="79"/>
+      <c r="F6" s="79"/>
+      <c r="G6" s="79"/>
+      <c r="H6" s="79"/>
+      <c r="I6" s="79"/>
+      <c r="J6" s="79"/>
+      <c r="K6" s="80"/>
       <c r="L6" s="8"/>
     </row>
-    <row r="7" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="69"/>
-      <c r="B7" s="44" t="s">
+    <row r="7" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="24"/>
+      <c r="B7" s="68" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
-      <c r="G7" s="46"/>
-      <c r="H7" s="53"/>
-      <c r="I7" s="35" t="s">
+      <c r="C7" s="69"/>
+      <c r="D7" s="69"/>
+      <c r="E7" s="69"/>
+      <c r="F7" s="69"/>
+      <c r="G7" s="70"/>
+      <c r="H7" s="77"/>
+      <c r="I7" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="J7" s="36"/>
-      <c r="K7" s="36"/>
-      <c r="L7" s="36"/>
-      <c r="M7" s="36"/>
-      <c r="N7" s="37"/>
-      <c r="O7" s="54"/>
-      <c r="P7" s="24"/>
-      <c r="Q7" s="25"/>
-      <c r="R7" s="69"/>
+      <c r="J7" s="60"/>
+      <c r="K7" s="60"/>
+      <c r="L7" s="60"/>
+      <c r="M7" s="60"/>
+      <c r="N7" s="61"/>
+      <c r="O7" s="30"/>
+      <c r="P7" s="48"/>
+      <c r="Q7" s="49"/>
+      <c r="R7" s="24"/>
       <c r="S7" s="2"/>
       <c r="T7" s="2"/>
     </row>
-    <row r="8" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="70"/>
-      <c r="B8" s="47"/>
-      <c r="C8" s="48"/>
-      <c r="D8" s="48"/>
-      <c r="E8" s="48"/>
-      <c r="F8" s="48"/>
-      <c r="G8" s="49"/>
-      <c r="H8" s="54"/>
-      <c r="I8" s="38"/>
-      <c r="J8" s="39"/>
-      <c r="K8" s="39"/>
-      <c r="L8" s="39"/>
-      <c r="M8" s="39"/>
-      <c r="N8" s="40"/>
-      <c r="O8" s="54"/>
-      <c r="P8" s="26"/>
-      <c r="Q8" s="27"/>
-      <c r="R8" s="70"/>
+    <row r="8" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="25"/>
+      <c r="B8" s="71"/>
+      <c r="C8" s="72"/>
+      <c r="D8" s="72"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="73"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="62"/>
+      <c r="J8" s="63"/>
+      <c r="K8" s="63"/>
+      <c r="L8" s="63"/>
+      <c r="M8" s="63"/>
+      <c r="N8" s="64"/>
+      <c r="O8" s="30"/>
+      <c r="P8" s="50"/>
+      <c r="Q8" s="51"/>
+      <c r="R8" s="25"/>
       <c r="S8" s="2"/>
       <c r="T8" s="2"/>
     </row>
-    <row r="9" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="71"/>
-      <c r="B9" s="50"/>
-      <c r="C9" s="51"/>
-      <c r="D9" s="51"/>
-      <c r="E9" s="51"/>
-      <c r="F9" s="51"/>
-      <c r="G9" s="52"/>
-      <c r="H9" s="54"/>
-      <c r="I9" s="41"/>
-      <c r="J9" s="42"/>
-      <c r="K9" s="42"/>
-      <c r="L9" s="42"/>
-      <c r="M9" s="42"/>
-      <c r="N9" s="43"/>
-      <c r="O9" s="54"/>
-      <c r="P9" s="28"/>
-      <c r="Q9" s="29"/>
-      <c r="R9" s="71"/>
+    <row r="9" spans="1:22" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="26"/>
+      <c r="B9" s="74"/>
+      <c r="C9" s="75"/>
+      <c r="D9" s="75"/>
+      <c r="E9" s="75"/>
+      <c r="F9" s="75"/>
+      <c r="G9" s="76"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="65"/>
+      <c r="J9" s="66"/>
+      <c r="K9" s="66"/>
+      <c r="L9" s="66"/>
+      <c r="M9" s="66"/>
+      <c r="N9" s="67"/>
+      <c r="O9" s="30"/>
+      <c r="P9" s="52"/>
+      <c r="Q9" s="53"/>
+      <c r="R9" s="26"/>
       <c r="S9" s="2"/>
       <c r="T9" s="2"/>
     </row>
-    <row r="10" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="72" t="s">
+    <row r="10" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="81" t="s">
+      <c r="B10" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="82"/>
-      <c r="D10" s="75" t="s">
+      <c r="C10" s="41"/>
+      <c r="D10" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="76"/>
-      <c r="F10" s="75" t="s">
+      <c r="E10" s="33"/>
+      <c r="F10" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="G10" s="76"/>
-      <c r="H10" s="54"/>
-      <c r="I10" s="79" t="s">
+      <c r="G10" s="33"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="J10" s="80"/>
-      <c r="K10" s="79" t="s">
+      <c r="J10" s="37"/>
+      <c r="K10" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="L10" s="80"/>
-      <c r="M10" s="79" t="s">
+      <c r="L10" s="37"/>
+      <c r="M10" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="N10" s="80"/>
-      <c r="O10" s="54"/>
-      <c r="P10" s="63" t="s">
+      <c r="N10" s="37"/>
+      <c r="O10" s="30"/>
+      <c r="P10" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="Q10" s="64"/>
-      <c r="R10" s="72" t="s">
+      <c r="Q10" s="45"/>
+      <c r="R10" s="27" t="s">
         <v>3</v>
       </c>
       <c r="S10" s="21"/>
       <c r="T10" s="21"/>
-      <c r="U10" s="19" t="s">
+      <c r="U10" s="19"/>
+      <c r="V10" s="19" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="73"/>
-      <c r="B11" s="59" t="s">
+    <row r="11" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="28"/>
+      <c r="B11" s="81" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="60"/>
-      <c r="D11" s="77" t="s">
+      <c r="C11" s="82"/>
+      <c r="D11" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="78"/>
-      <c r="F11" s="77" t="s">
+      <c r="E11" s="35"/>
+      <c r="F11" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="G11" s="78"/>
-      <c r="H11" s="54"/>
-      <c r="I11" s="67" t="s">
+      <c r="G11" s="35"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="J11" s="68"/>
-      <c r="K11" s="67" t="s">
+      <c r="J11" s="39"/>
+      <c r="K11" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="L11" s="68"/>
-      <c r="M11" s="67" t="s">
+      <c r="L11" s="39"/>
+      <c r="M11" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="N11" s="68"/>
-      <c r="O11" s="54"/>
-      <c r="P11" s="65" t="s">
+      <c r="N11" s="39"/>
+      <c r="O11" s="30"/>
+      <c r="P11" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="Q11" s="66"/>
-      <c r="R11" s="73"/>
+      <c r="Q11" s="47"/>
+      <c r="R11" s="28"/>
       <c r="S11" s="21"/>
       <c r="T11" s="21"/>
     </row>
-    <row r="12" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="74"/>
+    <row r="12" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="29"/>
       <c r="B12" s="1" t="s">
         <v>4</v>
       </c>
@@ -1345,7 +1346,7 @@
       <c r="G12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H12" s="54"/>
+      <c r="H12" s="30"/>
       <c r="I12" s="1" t="s">
         <v>4</v>
       </c>
@@ -1364,18 +1365,18 @@
       <c r="N12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="O12" s="54"/>
+      <c r="O12" s="30"/>
       <c r="P12" s="5" t="s">
         <v>4</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="R12" s="74"/>
+      <c r="R12" s="29"/>
       <c r="S12" s="21"/>
       <c r="T12" s="21"/>
     </row>
-    <row r="13" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>1</v>
       </c>
@@ -1389,7 +1390,7 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
-      <c r="H13" s="54"/>
+      <c r="H13" s="30"/>
       <c r="I13" s="4" t="s">
         <v>18</v>
       </c>
@@ -1406,7 +1407,7 @@
       <c r="N13" s="4">
         <v>44.9</v>
       </c>
-      <c r="O13" s="54"/>
+      <c r="O13" s="30"/>
       <c r="P13" s="6">
         <f>SUM(B13+K13+M13)</f>
         <v>153.4</v>
@@ -1433,7 +1434,7 @@
         <v>329810</v>
       </c>
     </row>
-    <row r="14" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>2</v>
       </c>
@@ -1447,7 +1448,7 @@
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
-      <c r="H14" s="55"/>
+      <c r="H14" s="31"/>
       <c r="I14" s="4" t="s">
         <v>18</v>
       </c>
@@ -1462,7 +1463,7 @@
       </c>
       <c r="M14" s="4"/>
       <c r="N14" s="4"/>
-      <c r="O14" s="55"/>
+      <c r="O14" s="31"/>
       <c r="P14" s="6">
         <f>SUM(B14+K14)</f>
         <v>101.2</v>
@@ -1489,7 +1490,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="15" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>3</v>
       </c>
@@ -1541,7 +1542,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="16" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>4</v>
       </c>
@@ -1593,7 +1594,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="17" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>5</v>
       </c>
@@ -1645,7 +1646,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="18" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>6</v>
       </c>
@@ -1697,7 +1698,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="19" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>7</v>
       </c>
@@ -1749,7 +1750,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="20" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>8</v>
       </c>
@@ -1801,7 +1802,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="21" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>9</v>
       </c>
@@ -1853,7 +1854,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="22" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>10</v>
       </c>
@@ -1905,7 +1906,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="23" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>11</v>
       </c>
@@ -1957,7 +1958,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="24" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>12</v>
       </c>
@@ -2013,7 +2014,7 @@
         <v>766689.99999999988</v>
       </c>
     </row>
-    <row r="25" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>13</v>
       </c>
@@ -2065,7 +2066,7 @@
         <v>656180</v>
       </c>
     </row>
-    <row r="26" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>14</v>
       </c>
@@ -2121,7 +2122,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="27" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>15</v>
       </c>
@@ -2177,7 +2178,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="28" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>16</v>
       </c>
@@ -2233,7 +2234,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="29" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>17</v>
       </c>
@@ -2289,7 +2290,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="30" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>18</v>
       </c>
@@ -2345,7 +2346,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="31" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>19</v>
       </c>
@@ -2401,7 +2402,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="32" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>20</v>
       </c>
@@ -2457,7 +2458,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="33" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>21</v>
       </c>
@@ -2513,7 +2514,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="34" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>22</v>
       </c>
@@ -2569,7 +2570,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="35" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>23</v>
       </c>
@@ -2625,7 +2626,7 @@
         <v>231300</v>
       </c>
     </row>
-    <row r="36" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>24</v>
       </c>
@@ -2681,7 +2682,7 @@
         <v>231300</v>
       </c>
     </row>
-    <row r="37" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>25</v>
       </c>
@@ -2737,7 +2738,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="38" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>26</v>
       </c>
@@ -2793,7 +2794,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="39" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>27</v>
       </c>
@@ -2849,7 +2850,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="40" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>28</v>
       </c>
@@ -2905,7 +2906,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="41" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>29</v>
       </c>
@@ -2961,7 +2962,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="42" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>30</v>
       </c>
@@ -3017,7 +3018,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="43" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>31</v>
       </c>
@@ -3073,7 +3074,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="44" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>32</v>
       </c>
@@ -3129,7 +3130,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="45" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>33</v>
       </c>
@@ -3185,7 +3186,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="46" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>34</v>
       </c>
@@ -3237,7 +3238,7 @@
         <v>656180</v>
       </c>
     </row>
-    <row r="47" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>35</v>
       </c>
@@ -3289,7 +3290,7 @@
         <v>656180</v>
       </c>
     </row>
-    <row r="48" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>36</v>
       </c>
@@ -3345,7 +3346,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="49" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>37</v>
       </c>
@@ -3401,7 +3402,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="50" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>38</v>
       </c>
@@ -3457,7 +3458,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="51" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>39</v>
       </c>
@@ -3513,7 +3514,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="52" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>40</v>
       </c>
@@ -3569,7 +3570,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="53" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
         <v>41</v>
       </c>
@@ -3625,7 +3626,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="54" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1">
         <v>42</v>
       </c>
@@ -3681,7 +3682,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="55" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1">
         <v>43</v>
       </c>
@@ -3737,7 +3738,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="56" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1">
         <v>44</v>
       </c>
@@ -3793,7 +3794,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="57" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1">
         <v>45</v>
       </c>
@@ -3849,7 +3850,7 @@
         <v>231300</v>
       </c>
     </row>
-    <row r="58" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1">
         <v>46</v>
       </c>
@@ -3905,7 +3906,7 @@
         <v>231300</v>
       </c>
     </row>
-    <row r="59" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1">
         <v>47</v>
       </c>
@@ -3961,7 +3962,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="60" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1">
         <v>48</v>
       </c>
@@ -4017,7 +4018,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="61" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1">
         <v>49</v>
       </c>
@@ -4073,7 +4074,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="62" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1">
         <v>50</v>
       </c>
@@ -4129,7 +4130,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="63" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1">
         <v>51</v>
       </c>
@@ -4185,7 +4186,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="64" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1">
         <v>52</v>
       </c>
@@ -4241,7 +4242,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="65" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1">
         <v>53</v>
       </c>
@@ -4297,7 +4298,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="66" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1">
         <v>54</v>
       </c>
@@ -4353,7 +4354,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="67" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1">
         <v>55</v>
       </c>
@@ -4409,7 +4410,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="68" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1">
         <v>56</v>
       </c>
@@ -4461,7 +4462,7 @@
         <v>656180</v>
       </c>
     </row>
-    <row r="69" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1">
         <v>57</v>
       </c>
@@ -4517,7 +4518,7 @@
         <v>903645</v>
       </c>
     </row>
-    <row r="70" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1">
         <v>58</v>
       </c>
@@ -4569,7 +4570,7 @@
         <v>284400</v>
       </c>
     </row>
-    <row r="71" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="1">
         <v>59</v>
       </c>
@@ -4621,7 +4622,7 @@
         <v>284400</v>
       </c>
     </row>
-    <row r="72" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="1">
         <v>60</v>
       </c>
@@ -4673,7 +4674,7 @@
         <v>284400</v>
       </c>
     </row>
-    <row r="73" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="1">
         <v>61</v>
       </c>
@@ -4725,7 +4726,7 @@
         <v>284400</v>
       </c>
     </row>
-    <row r="74" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="1">
         <v>62</v>
       </c>
@@ -4777,7 +4778,7 @@
         <v>284400</v>
       </c>
     </row>
-    <row r="75" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1">
         <v>63</v>
       </c>
@@ -4829,7 +4830,7 @@
         <v>284400</v>
       </c>
     </row>
-    <row r="76" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="1">
         <v>64</v>
       </c>
@@ -4881,7 +4882,7 @@
         <v>284400</v>
       </c>
     </row>
-    <row r="77" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="1">
         <v>65</v>
       </c>
@@ -4933,7 +4934,7 @@
         <v>284400</v>
       </c>
     </row>
-    <row r="78" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="1">
         <v>66</v>
       </c>
@@ -4985,7 +4986,7 @@
         <v>284400</v>
       </c>
     </row>
-    <row r="79" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="1">
         <v>67</v>
       </c>
@@ -5037,7 +5038,7 @@
         <v>276060</v>
       </c>
     </row>
-    <row r="80" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:22" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="1">
         <v>68</v>
       </c>
@@ -5089,7 +5090,7 @@
         <v>231300</v>
       </c>
     </row>
-    <row r="81" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="1">
         <v>69</v>
       </c>
@@ -5141,7 +5142,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="82" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="1">
         <v>70</v>
       </c>
@@ -5193,7 +5194,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="83" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="1">
         <v>71</v>
       </c>
@@ -5245,7 +5246,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="84" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="1">
         <v>72</v>
       </c>
@@ -5297,7 +5298,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="85" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="1">
         <v>73</v>
       </c>
@@ -5349,7 +5350,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="86" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="1">
         <v>74</v>
       </c>
@@ -5401,7 +5402,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="87" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="1">
         <v>75</v>
       </c>
@@ -5453,7 +5454,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="88" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="1">
         <v>76</v>
       </c>
@@ -5505,7 +5506,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="89" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="1">
         <v>77</v>
       </c>
@@ -5557,7 +5558,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="90" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="1">
         <v>78</v>
       </c>
@@ -5609,7 +5610,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="91" spans="1:23" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:23" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A91" s="1">
         <v>79</v>
       </c>
@@ -5661,7 +5662,7 @@
         <v>227700</v>
       </c>
     </row>
-    <row r="92" spans="1:23" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:23" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A92" s="2"/>
       <c r="H92"/>
       <c r="O92"/>
@@ -5673,7 +5674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:23" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="9"/>
       <c r="B93" s="14"/>
       <c r="C93" s="14"/>
@@ -5695,11 +5696,11 @@
       <c r="Q93" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="R93" s="69"/>
+      <c r="R93" s="24"/>
       <c r="S93" s="2"/>
       <c r="T93" s="22"/>
     </row>
-    <row r="94" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A94" s="17" t="s">
         <v>20</v>
       </c>
@@ -5716,19 +5717,19 @@
       <c r="L94" s="13"/>
       <c r="M94" s="13"/>
       <c r="N94" s="18"/>
-      <c r="P94" s="61">
+      <c r="P94" s="42">
         <f>SUM(P13:P91)</f>
         <v>9699.4999999999982</v>
       </c>
-      <c r="Q94" s="61">
+      <c r="Q94" s="42">
         <f>SUM(Q13:Q91)</f>
         <v>8964.8999999999978</v>
       </c>
-      <c r="R94" s="70"/>
+      <c r="R94" s="25"/>
       <c r="S94" s="2"/>
       <c r="T94" s="22"/>
     </row>
-    <row r="95" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="10"/>
       <c r="B95" s="11"/>
       <c r="C95" s="11"/>
@@ -5743,9 +5744,9 @@
       <c r="L95" s="11"/>
       <c r="M95" s="11"/>
       <c r="N95" s="12"/>
-      <c r="P95" s="62"/>
-      <c r="Q95" s="62"/>
-      <c r="R95" s="71"/>
+      <c r="P95" s="43"/>
+      <c r="Q95" s="43"/>
+      <c r="R95" s="26"/>
       <c r="S95" s="2"/>
       <c r="T95" s="22"/>
       <c r="U95" s="7">
@@ -5761,7 +5762,7 @@
         <v>2196925</v>
       </c>
     </row>
-    <row r="96" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:23" x14ac:dyDescent="0.2">
       <c r="T96" s="22"/>
       <c r="V96" s="23">
         <f>(V95-U95)/V95</f>
@@ -5770,6 +5771,25 @@
     </row>
   </sheetData>
   <mergeCells count="35">
+    <mergeCell ref="P7:Q9"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C1:K1"/>
+    <mergeCell ref="C2:N2"/>
+    <mergeCell ref="C3:M3"/>
+    <mergeCell ref="C4:M4"/>
+    <mergeCell ref="I7:N9"/>
+    <mergeCell ref="B7:G9"/>
+    <mergeCell ref="H7:H14"/>
+    <mergeCell ref="A6:K6"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="P94:P95"/>
+    <mergeCell ref="Q94:Q95"/>
+    <mergeCell ref="P10:Q10"/>
+    <mergeCell ref="P11:Q11"/>
+    <mergeCell ref="M11:N11"/>
     <mergeCell ref="R93:R95"/>
     <mergeCell ref="A7:A9"/>
     <mergeCell ref="R7:R9"/>
@@ -5786,25 +5806,6 @@
     <mergeCell ref="M10:N10"/>
     <mergeCell ref="A10:A12"/>
     <mergeCell ref="B10:C10"/>
-    <mergeCell ref="P94:P95"/>
-    <mergeCell ref="Q94:Q95"/>
-    <mergeCell ref="P10:Q10"/>
-    <mergeCell ref="P11:Q11"/>
-    <mergeCell ref="M11:N11"/>
-    <mergeCell ref="P7:Q9"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C1:K1"/>
-    <mergeCell ref="C2:N2"/>
-    <mergeCell ref="C3:M3"/>
-    <mergeCell ref="C4:M4"/>
-    <mergeCell ref="I7:N9"/>
-    <mergeCell ref="B7:G9"/>
-    <mergeCell ref="H7:H14"/>
-    <mergeCell ref="A6:K6"/>
-    <mergeCell ref="B11:C11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
@@ -5821,7 +5822,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5830,7 +5831,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>